<commit_message>
watchlist: agregar AGRO.BA (alta manual desde la app)
</commit_message>
<xml_diff>
--- a/data/tickers.xlsx
+++ b/data/tickers.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A994"/>
+  <dimension ref="A1:A995"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5369,9 +5369,14 @@
         <v/>
       </c>
     </row>
+    <row r="995">
+      <c r="A995" t="str">
+        <v>AGRO.BA</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A994"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A995"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
watchlist: agregar SEMI.BA (alta manual desde la app)
</commit_message>
<xml_diff>
--- a/data/tickers.xlsx
+++ b/data/tickers.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A995"/>
+  <dimension ref="A1:A996"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5374,9 +5374,14 @@
         <v>AGRO.BA</v>
       </c>
     </row>
+    <row r="996">
+      <c r="A996" t="str">
+        <v>SEMI.BA</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A995"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A996"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
watchlist: eliminar CELU (baja manual desde la app)
</commit_message>
<xml_diff>
--- a/data/tickers.xlsx
+++ b/data/tickers.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A996"/>
+  <dimension ref="A1:A995"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2246,302 +2246,302 @@
     </row>
     <row r="370">
       <c r="A370" t="str">
-        <v>CELU</v>
+        <v>CECO2</v>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="str">
-        <v>CECO2</v>
+        <v>ETHA</v>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="str">
-        <v>ETHA</v>
+        <v>IBIT</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="str">
-        <v>IBIT</v>
+        <v>LAC</v>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="str">
-        <v>LAC</v>
+        <v>DIVIDENDOS</v>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="str">
-        <v>DIVIDENDOS</v>
+        <v>PNZIF</v>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="str">
-        <v>PNZIF</v>
+        <v>ASML</v>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="str">
-        <v>ASML</v>
+        <v>TEAM</v>
       </c>
     </row>
     <row r="378">
       <c r="A378" t="str">
-        <v>TEAM</v>
+        <v>AI</v>
       </c>
     </row>
     <row r="379">
       <c r="A379" t="str">
-        <v>AI</v>
+        <v>CLS</v>
       </c>
     </row>
     <row r="380">
       <c r="A380" t="str">
-        <v>CLS</v>
+        <v>CEG</v>
       </c>
     </row>
     <row r="381">
       <c r="A381" t="str">
-        <v>CEG</v>
+        <v>DECK</v>
       </c>
     </row>
     <row r="382">
       <c r="A382" t="str">
-        <v>DECK</v>
+        <v>RGTI</v>
       </c>
     </row>
     <row r="383">
       <c r="A383" t="str">
-        <v>RGTI</v>
+        <v>NOW</v>
       </c>
     </row>
     <row r="384">
       <c r="A384" t="str">
-        <v>NOW</v>
+        <v>TEM</v>
       </c>
     </row>
     <row r="385">
       <c r="A385" t="str">
-        <v>TEM</v>
+        <v>PATH</v>
       </c>
     </row>
     <row r="386">
       <c r="A386" t="str">
-        <v>PATH</v>
+        <v>VRTX</v>
       </c>
     </row>
     <row r="387">
       <c r="A387" t="str">
-        <v>VRTX</v>
+        <v>VST</v>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="str">
-        <v>VST</v>
+        <v>USO</v>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="str">
-        <v>USO</v>
+        <v>EFA</v>
       </c>
     </row>
     <row r="390">
       <c r="A390" t="str">
-        <v>EFA</v>
+        <v>IEMG</v>
       </c>
     </row>
     <row r="391">
       <c r="A391" t="str">
-        <v>IEMG</v>
+        <v>ACWI</v>
       </c>
     </row>
     <row r="392">
       <c r="A392" t="str">
-        <v>ACWI</v>
+        <v>GDX</v>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="str">
-        <v>GDX</v>
+        <v>HOOD</v>
       </c>
     </row>
     <row r="394">
       <c r="A394" t="str">
-        <v>HOOD</v>
+        <v>CRWV</v>
       </c>
     </row>
     <row r="395">
       <c r="A395" t="str">
-        <v>CRWV</v>
+        <v>OKLO</v>
       </c>
     </row>
     <row r="396">
       <c r="A396" t="str">
-        <v>OKLO</v>
+        <v>RKLB</v>
       </c>
     </row>
     <row r="397">
       <c r="A397" t="str">
-        <v>RKLB</v>
+        <v>ALAB</v>
       </c>
     </row>
     <row r="398">
       <c r="A398" t="str">
-        <v>ALAB</v>
+        <v>ASTS</v>
       </c>
     </row>
     <row r="399">
       <c r="A399" t="str">
-        <v>ASTS</v>
+        <v>IREN</v>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="str">
-        <v>IREN</v>
+        <v>ECL</v>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="str">
-        <v>ECL</v>
+        <v>SPHQ</v>
       </c>
     </row>
     <row r="402">
       <c r="A402" t="str">
-        <v>SPHQ</v>
+        <v>EFECTIVO</v>
       </c>
     </row>
     <row r="403">
       <c r="A403" t="str">
-        <v>EFECTIVO</v>
+        <v>URA</v>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="str">
-        <v>URA</v>
+        <v>COPX</v>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="str">
-        <v>COPX</v>
+        <v>ILF</v>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="str">
-        <v>ILF</v>
+        <v>ESGU</v>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="str">
-        <v>ESGU</v>
+        <v>IVV</v>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="str">
-        <v>IVV</v>
+        <v>BMNR</v>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="str">
-        <v>BMNR</v>
+        <v>BX</v>
       </c>
     </row>
     <row r="410">
       <c r="A410" t="str">
-        <v>BX</v>
+        <v>RSP</v>
       </c>
     </row>
     <row r="411">
       <c r="A411" t="str">
-        <v>RSP</v>
+        <v>EWI</v>
       </c>
     </row>
     <row r="412">
       <c r="A412" t="str">
-        <v>EWI</v>
+        <v>XME</v>
       </c>
     </row>
     <row r="413">
       <c r="A413" t="str">
-        <v>XME</v>
+        <v>ICLN</v>
       </c>
     </row>
     <row r="414">
       <c r="A414" t="str">
-        <v>ICLN</v>
+        <v>CRWD</v>
       </c>
     </row>
     <row r="415">
       <c r="A415" t="str">
-        <v>CRWD</v>
+        <v>ANET</v>
       </c>
     </row>
     <row r="416">
       <c r="A416" t="str">
-        <v>ANET</v>
+        <v>O</v>
       </c>
     </row>
     <row r="417">
       <c r="A417" t="str">
-        <v>O</v>
+        <v>GLNG</v>
       </c>
     </row>
     <row r="418">
       <c r="A418" t="str">
-        <v>GLNG</v>
+        <v>SNDK</v>
       </c>
     </row>
     <row r="419">
       <c r="A419" t="str">
-        <v>SNDK</v>
+        <v>NBIS</v>
       </c>
     </row>
     <row r="420">
       <c r="A420" t="str">
-        <v>NBIS</v>
+        <v>HIMS</v>
       </c>
     </row>
     <row r="421">
       <c r="A421" t="str">
-        <v>HIMS</v>
+        <v>ONDS</v>
       </c>
     </row>
     <row r="422">
       <c r="A422" t="str">
-        <v>ONDS</v>
+        <v>COP</v>
       </c>
     </row>
     <row r="423">
       <c r="A423" t="str">
-        <v>COP</v>
+        <v>NEE</v>
       </c>
     </row>
     <row r="424">
       <c r="A424" t="str">
-        <v>NEE</v>
+        <v>MP</v>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="str">
-        <v>MP</v>
+        <v>CCJ</v>
       </c>
     </row>
     <row r="426">
       <c r="A426" t="str">
-        <v>CCJ</v>
+        <v>FISV</v>
       </c>
     </row>
     <row r="427">
       <c r="A427" t="str">
-        <v>FISV</v>
+        <v>KEEL</v>
       </c>
     </row>
     <row r="428">
       <c r="A428" t="str">
-        <v>KEEL</v>
+        <v>NVO</v>
       </c>
     </row>
     <row r="429">
       <c r="A429" t="str">
-        <v>NVO</v>
+        <v/>
       </c>
     </row>
     <row r="430">
@@ -5366,22 +5366,17 @@
     </row>
     <row r="994">
       <c r="A994" t="str">
-        <v/>
+        <v>AGRO.BA</v>
       </c>
     </row>
     <row r="995">
       <c r="A995" t="str">
-        <v>AGRO.BA</v>
-      </c>
-    </row>
-    <row r="996">
-      <c r="A996" t="str">
         <v>SEMI.BA</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A996"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A995"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
watchlist: agregar EWY (alta manual desde la app)
</commit_message>
<xml_diff>
--- a/data/tickers.xlsx
+++ b/data/tickers.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A995"/>
+  <dimension ref="A1:A996"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5374,9 +5374,14 @@
         <v>SEMI.BA</v>
       </c>
     </row>
+    <row r="996">
+      <c r="A996" t="str">
+        <v>EWY</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A995"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A996"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
watchlist: agregar SPCX (alta manual desde la app)
</commit_message>
<xml_diff>
--- a/data/tickers.xlsx
+++ b/data/tickers.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A996"/>
+  <dimension ref="A1:A997"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5379,9 +5379,14 @@
         <v>EWY</v>
       </c>
     </row>
+    <row r="997">
+      <c r="A997" t="str">
+        <v>SPCX</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A996"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A997"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
watchlist: eliminar TRVV (baja manual desde la app)
</commit_message>
<xml_diff>
--- a/data/tickers.xlsx
+++ b/data/tickers.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A995"/>
+  <dimension ref="A1:A994"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2076,457 +2076,457 @@
     </row>
     <row r="336">
       <c r="A336" t="str">
-        <v>TRVV</v>
+        <v>TSMC</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="str">
-        <v>TSMC</v>
+        <v>TTM</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="str">
-        <v>TTM</v>
+        <v>TV</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="str">
-        <v>TV</v>
+        <v>TWTR</v>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="str">
-        <v>TWTR</v>
+        <v>TXR</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="str">
-        <v>TXR</v>
+        <v>VALO</v>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="str">
-        <v>VALO</v>
+        <v>WBA</v>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="str">
-        <v>WBA</v>
+        <v>WBO</v>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="str">
-        <v>WBO</v>
+        <v>XROX</v>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="str">
-        <v>XROX</v>
+        <v>YPFD</v>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="str">
-        <v>YPFD</v>
+        <v>YZCA</v>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="str">
-        <v>YZCA</v>
+        <v>EQNR</v>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="str">
-        <v>EQNR</v>
+        <v>ARM</v>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="str">
-        <v>ARM</v>
+        <v>BKR</v>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="str">
-        <v>BKR</v>
+        <v>DHR</v>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="str">
-        <v>DHR</v>
+        <v>GT</v>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="str">
-        <v>GT</v>
+        <v>ISRG</v>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="str">
-        <v>ISRG</v>
+        <v>LAAC</v>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="str">
-        <v>LAAC</v>
+        <v>NXE</v>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="str">
-        <v>NXE</v>
+        <v>ORLY</v>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="str">
-        <v>ORLY</v>
+        <v>TJX</v>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="str">
-        <v>TJX</v>
+        <v>SAMI</v>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="str">
-        <v>SAMI</v>
+        <v>BHIP</v>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="str">
-        <v>BHIP</v>
+        <v>SEMI</v>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="str">
-        <v>SEMI</v>
+        <v>FERR</v>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="str">
-        <v>FERR</v>
+        <v>AGRO</v>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="str">
-        <v>AGRO</v>
+        <v>IRS</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="str">
-        <v>IRS</v>
+        <v>AL 30</v>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="str">
-        <v>AL 30</v>
+        <v>GD 30</v>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="str">
-        <v>GD 30</v>
+        <v>AL 29</v>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="str">
-        <v>AL 29</v>
+        <v>GD29</v>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="str">
-        <v>GD29</v>
+        <v>CECO2</v>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="str">
-        <v>CECO2</v>
+        <v>ETHA</v>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="str">
-        <v>ETHA</v>
+        <v>IBIT</v>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="str">
-        <v>IBIT</v>
+        <v>LAC</v>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="str">
-        <v>LAC</v>
+        <v>DIVIDENDOS</v>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="str">
-        <v>DIVIDENDOS</v>
+        <v>PNZIF</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="str">
-        <v>PNZIF</v>
+        <v>ASML</v>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="str">
-        <v>ASML</v>
+        <v>TEAM</v>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="str">
-        <v>TEAM</v>
+        <v>AI</v>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="str">
-        <v>AI</v>
+        <v>CLS</v>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="str">
-        <v>CLS</v>
+        <v>CEG</v>
       </c>
     </row>
     <row r="378">
       <c r="A378" t="str">
-        <v>CEG</v>
+        <v>DECK</v>
       </c>
     </row>
     <row r="379">
       <c r="A379" t="str">
-        <v>DECK</v>
+        <v>RGTI</v>
       </c>
     </row>
     <row r="380">
       <c r="A380" t="str">
-        <v>RGTI</v>
+        <v>NOW</v>
       </c>
     </row>
     <row r="381">
       <c r="A381" t="str">
-        <v>NOW</v>
+        <v>TEM</v>
       </c>
     </row>
     <row r="382">
       <c r="A382" t="str">
-        <v>TEM</v>
+        <v>PATH</v>
       </c>
     </row>
     <row r="383">
       <c r="A383" t="str">
-        <v>PATH</v>
+        <v>VRTX</v>
       </c>
     </row>
     <row r="384">
       <c r="A384" t="str">
-        <v>VRTX</v>
+        <v>VST</v>
       </c>
     </row>
     <row r="385">
       <c r="A385" t="str">
-        <v>VST</v>
+        <v>USO</v>
       </c>
     </row>
     <row r="386">
       <c r="A386" t="str">
-        <v>USO</v>
+        <v>EFA</v>
       </c>
     </row>
     <row r="387">
       <c r="A387" t="str">
-        <v>EFA</v>
+        <v>IEMG</v>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="str">
-        <v>IEMG</v>
+        <v>ACWI</v>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="str">
-        <v>ACWI</v>
+        <v>GDX</v>
       </c>
     </row>
     <row r="390">
       <c r="A390" t="str">
-        <v>GDX</v>
+        <v>HOOD</v>
       </c>
     </row>
     <row r="391">
       <c r="A391" t="str">
-        <v>HOOD</v>
+        <v>CRWV</v>
       </c>
     </row>
     <row r="392">
       <c r="A392" t="str">
-        <v>CRWV</v>
+        <v>OKLO</v>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="str">
-        <v>OKLO</v>
+        <v>RKLB</v>
       </c>
     </row>
     <row r="394">
       <c r="A394" t="str">
-        <v>RKLB</v>
+        <v>ALAB</v>
       </c>
     </row>
     <row r="395">
       <c r="A395" t="str">
-        <v>ALAB</v>
+        <v>ASTS</v>
       </c>
     </row>
     <row r="396">
       <c r="A396" t="str">
-        <v>ASTS</v>
+        <v>IREN</v>
       </c>
     </row>
     <row r="397">
       <c r="A397" t="str">
-        <v>IREN</v>
+        <v>ECL</v>
       </c>
     </row>
     <row r="398">
       <c r="A398" t="str">
-        <v>ECL</v>
+        <v>SPHQ</v>
       </c>
     </row>
     <row r="399">
       <c r="A399" t="str">
-        <v>SPHQ</v>
+        <v>EFECTIVO</v>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="str">
-        <v>EFECTIVO</v>
+        <v>URA</v>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="str">
-        <v>URA</v>
+        <v>COPX</v>
       </c>
     </row>
     <row r="402">
       <c r="A402" t="str">
-        <v>COPX</v>
+        <v>ILF</v>
       </c>
     </row>
     <row r="403">
       <c r="A403" t="str">
-        <v>ILF</v>
+        <v>ESGU</v>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="str">
-        <v>ESGU</v>
+        <v>IVV</v>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="str">
-        <v>IVV</v>
+        <v>BMNR</v>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="str">
-        <v>BMNR</v>
+        <v>BX</v>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="str">
-        <v>BX</v>
+        <v>RSP</v>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="str">
-        <v>RSP</v>
+        <v>EWI</v>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="str">
-        <v>EWI</v>
+        <v>XME</v>
       </c>
     </row>
     <row r="410">
       <c r="A410" t="str">
-        <v>XME</v>
+        <v>ICLN</v>
       </c>
     </row>
     <row r="411">
       <c r="A411" t="str">
-        <v>ICLN</v>
+        <v>CRWD</v>
       </c>
     </row>
     <row r="412">
       <c r="A412" t="str">
-        <v>CRWD</v>
+        <v>ANET</v>
       </c>
     </row>
     <row r="413">
       <c r="A413" t="str">
-        <v>ANET</v>
+        <v>O</v>
       </c>
     </row>
     <row r="414">
       <c r="A414" t="str">
-        <v>O</v>
+        <v>GLNG</v>
       </c>
     </row>
     <row r="415">
       <c r="A415" t="str">
-        <v>GLNG</v>
+        <v>SNDK</v>
       </c>
     </row>
     <row r="416">
       <c r="A416" t="str">
-        <v>SNDK</v>
+        <v>NBIS</v>
       </c>
     </row>
     <row r="417">
       <c r="A417" t="str">
-        <v>NBIS</v>
+        <v>HIMS</v>
       </c>
     </row>
     <row r="418">
       <c r="A418" t="str">
-        <v>HIMS</v>
+        <v>ONDS</v>
       </c>
     </row>
     <row r="419">
       <c r="A419" t="str">
-        <v>ONDS</v>
+        <v>COP</v>
       </c>
     </row>
     <row r="420">
       <c r="A420" t="str">
-        <v>COP</v>
+        <v>NEE</v>
       </c>
     </row>
     <row r="421">
       <c r="A421" t="str">
-        <v>NEE</v>
+        <v>MP</v>
       </c>
     </row>
     <row r="422">
       <c r="A422" t="str">
-        <v>MP</v>
+        <v>CCJ</v>
       </c>
     </row>
     <row r="423">
       <c r="A423" t="str">
-        <v>CCJ</v>
+        <v>FISV</v>
       </c>
     </row>
     <row r="424">
       <c r="A424" t="str">
-        <v>FISV</v>
+        <v>KEEL</v>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="str">
-        <v>KEEL</v>
+        <v>NVO</v>
       </c>
     </row>
     <row r="426">
       <c r="A426" t="str">
-        <v>NVO</v>
+        <v/>
       </c>
     </row>
     <row r="427">
@@ -5351,32 +5351,27 @@
     </row>
     <row r="991">
       <c r="A991" t="str">
-        <v/>
+        <v>AGRO.BA</v>
       </c>
     </row>
     <row r="992">
       <c r="A992" t="str">
-        <v>AGRO.BA</v>
+        <v>SEMI.BA</v>
       </c>
     </row>
     <row r="993">
       <c r="A993" t="str">
-        <v>SEMI.BA</v>
+        <v>EWY</v>
       </c>
     </row>
     <row r="994">
       <c r="A994" t="str">
-        <v>EWY</v>
-      </c>
-    </row>
-    <row r="995">
-      <c r="A995" t="str">
         <v>SPCX</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A995"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A994"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
watchlist: eliminar TTM (baja manual desde la app)
</commit_message>
<xml_diff>
--- a/data/tickers.xlsx
+++ b/data/tickers.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A994"/>
+  <dimension ref="A1:A993"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2081,447 +2081,447 @@
     </row>
     <row r="337">
       <c r="A337" t="str">
-        <v>TTM</v>
+        <v>TV</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="str">
-        <v>TV</v>
+        <v>TWTR</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="str">
-        <v>TWTR</v>
+        <v>TXR</v>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="str">
-        <v>TXR</v>
+        <v>VALO</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="str">
-        <v>VALO</v>
+        <v>WBA</v>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="str">
-        <v>WBA</v>
+        <v>WBO</v>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="str">
-        <v>WBO</v>
+        <v>XROX</v>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="str">
-        <v>XROX</v>
+        <v>YPFD</v>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="str">
-        <v>YPFD</v>
+        <v>YZCA</v>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="str">
-        <v>YZCA</v>
+        <v>EQNR</v>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="str">
-        <v>EQNR</v>
+        <v>ARM</v>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="str">
-        <v>ARM</v>
+        <v>BKR</v>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="str">
-        <v>BKR</v>
+        <v>DHR</v>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="str">
-        <v>DHR</v>
+        <v>GT</v>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="str">
-        <v>GT</v>
+        <v>ISRG</v>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="str">
-        <v>ISRG</v>
+        <v>LAAC</v>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="str">
-        <v>LAAC</v>
+        <v>NXE</v>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="str">
-        <v>NXE</v>
+        <v>ORLY</v>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="str">
-        <v>ORLY</v>
+        <v>TJX</v>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="str">
-        <v>TJX</v>
+        <v>SAMI</v>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="str">
-        <v>SAMI</v>
+        <v>BHIP</v>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="str">
-        <v>BHIP</v>
+        <v>SEMI</v>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="str">
-        <v>SEMI</v>
+        <v>FERR</v>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="str">
-        <v>FERR</v>
+        <v>AGRO</v>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="str">
-        <v>AGRO</v>
+        <v>IRS</v>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="str">
-        <v>IRS</v>
+        <v>AL 30</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="str">
-        <v>AL 30</v>
+        <v>GD 30</v>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="str">
-        <v>GD 30</v>
+        <v>AL 29</v>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="str">
-        <v>AL 29</v>
+        <v>GD29</v>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="str">
-        <v>GD29</v>
+        <v>CECO2</v>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="str">
-        <v>CECO2</v>
+        <v>ETHA</v>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="str">
-        <v>ETHA</v>
+        <v>IBIT</v>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="str">
-        <v>IBIT</v>
+        <v>LAC</v>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="str">
-        <v>LAC</v>
+        <v>DIVIDENDOS</v>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="str">
-        <v>DIVIDENDOS</v>
+        <v>PNZIF</v>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="str">
-        <v>PNZIF</v>
+        <v>ASML</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="str">
-        <v>ASML</v>
+        <v>TEAM</v>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="str">
-        <v>TEAM</v>
+        <v>AI</v>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="str">
-        <v>AI</v>
+        <v>CLS</v>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="str">
-        <v>CLS</v>
+        <v>CEG</v>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="str">
-        <v>CEG</v>
+        <v>DECK</v>
       </c>
     </row>
     <row r="378">
       <c r="A378" t="str">
-        <v>DECK</v>
+        <v>RGTI</v>
       </c>
     </row>
     <row r="379">
       <c r="A379" t="str">
-        <v>RGTI</v>
+        <v>NOW</v>
       </c>
     </row>
     <row r="380">
       <c r="A380" t="str">
-        <v>NOW</v>
+        <v>TEM</v>
       </c>
     </row>
     <row r="381">
       <c r="A381" t="str">
-        <v>TEM</v>
+        <v>PATH</v>
       </c>
     </row>
     <row r="382">
       <c r="A382" t="str">
-        <v>PATH</v>
+        <v>VRTX</v>
       </c>
     </row>
     <row r="383">
       <c r="A383" t="str">
-        <v>VRTX</v>
+        <v>VST</v>
       </c>
     </row>
     <row r="384">
       <c r="A384" t="str">
-        <v>VST</v>
+        <v>USO</v>
       </c>
     </row>
     <row r="385">
       <c r="A385" t="str">
-        <v>USO</v>
+        <v>EFA</v>
       </c>
     </row>
     <row r="386">
       <c r="A386" t="str">
-        <v>EFA</v>
+        <v>IEMG</v>
       </c>
     </row>
     <row r="387">
       <c r="A387" t="str">
-        <v>IEMG</v>
+        <v>ACWI</v>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="str">
-        <v>ACWI</v>
+        <v>GDX</v>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="str">
-        <v>GDX</v>
+        <v>HOOD</v>
       </c>
     </row>
     <row r="390">
       <c r="A390" t="str">
-        <v>HOOD</v>
+        <v>CRWV</v>
       </c>
     </row>
     <row r="391">
       <c r="A391" t="str">
-        <v>CRWV</v>
+        <v>OKLO</v>
       </c>
     </row>
     <row r="392">
       <c r="A392" t="str">
-        <v>OKLO</v>
+        <v>RKLB</v>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="str">
-        <v>RKLB</v>
+        <v>ALAB</v>
       </c>
     </row>
     <row r="394">
       <c r="A394" t="str">
-        <v>ALAB</v>
+        <v>ASTS</v>
       </c>
     </row>
     <row r="395">
       <c r="A395" t="str">
-        <v>ASTS</v>
+        <v>IREN</v>
       </c>
     </row>
     <row r="396">
       <c r="A396" t="str">
-        <v>IREN</v>
+        <v>ECL</v>
       </c>
     </row>
     <row r="397">
       <c r="A397" t="str">
-        <v>ECL</v>
+        <v>SPHQ</v>
       </c>
     </row>
     <row r="398">
       <c r="A398" t="str">
-        <v>SPHQ</v>
+        <v>EFECTIVO</v>
       </c>
     </row>
     <row r="399">
       <c r="A399" t="str">
-        <v>EFECTIVO</v>
+        <v>URA</v>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="str">
-        <v>URA</v>
+        <v>COPX</v>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="str">
-        <v>COPX</v>
+        <v>ILF</v>
       </c>
     </row>
     <row r="402">
       <c r="A402" t="str">
-        <v>ILF</v>
+        <v>ESGU</v>
       </c>
     </row>
     <row r="403">
       <c r="A403" t="str">
-        <v>ESGU</v>
+        <v>IVV</v>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="str">
-        <v>IVV</v>
+        <v>BMNR</v>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="str">
-        <v>BMNR</v>
+        <v>BX</v>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="str">
-        <v>BX</v>
+        <v>RSP</v>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="str">
-        <v>RSP</v>
+        <v>EWI</v>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="str">
-        <v>EWI</v>
+        <v>XME</v>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="str">
-        <v>XME</v>
+        <v>ICLN</v>
       </c>
     </row>
     <row r="410">
       <c r="A410" t="str">
-        <v>ICLN</v>
+        <v>CRWD</v>
       </c>
     </row>
     <row r="411">
       <c r="A411" t="str">
-        <v>CRWD</v>
+        <v>ANET</v>
       </c>
     </row>
     <row r="412">
       <c r="A412" t="str">
-        <v>ANET</v>
+        <v>O</v>
       </c>
     </row>
     <row r="413">
       <c r="A413" t="str">
-        <v>O</v>
+        <v>GLNG</v>
       </c>
     </row>
     <row r="414">
       <c r="A414" t="str">
-        <v>GLNG</v>
+        <v>SNDK</v>
       </c>
     </row>
     <row r="415">
       <c r="A415" t="str">
-        <v>SNDK</v>
+        <v>NBIS</v>
       </c>
     </row>
     <row r="416">
       <c r="A416" t="str">
-        <v>NBIS</v>
+        <v>HIMS</v>
       </c>
     </row>
     <row r="417">
       <c r="A417" t="str">
-        <v>HIMS</v>
+        <v>ONDS</v>
       </c>
     </row>
     <row r="418">
       <c r="A418" t="str">
-        <v>ONDS</v>
+        <v>COP</v>
       </c>
     </row>
     <row r="419">
       <c r="A419" t="str">
-        <v>COP</v>
+        <v>NEE</v>
       </c>
     </row>
     <row r="420">
       <c r="A420" t="str">
-        <v>NEE</v>
+        <v>MP</v>
       </c>
     </row>
     <row r="421">
       <c r="A421" t="str">
-        <v>MP</v>
+        <v>CCJ</v>
       </c>
     </row>
     <row r="422">
       <c r="A422" t="str">
-        <v>CCJ</v>
+        <v>FISV</v>
       </c>
     </row>
     <row r="423">
       <c r="A423" t="str">
-        <v>FISV</v>
+        <v>KEEL</v>
       </c>
     </row>
     <row r="424">
       <c r="A424" t="str">
-        <v>KEEL</v>
+        <v>NVO</v>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="str">
-        <v>NVO</v>
+        <v/>
       </c>
     </row>
     <row r="426">
@@ -5346,32 +5346,27 @@
     </row>
     <row r="990">
       <c r="A990" t="str">
-        <v/>
+        <v>AGRO.BA</v>
       </c>
     </row>
     <row r="991">
       <c r="A991" t="str">
-        <v>AGRO.BA</v>
+        <v>SEMI.BA</v>
       </c>
     </row>
     <row r="992">
       <c r="A992" t="str">
-        <v>SEMI.BA</v>
+        <v>EWY</v>
       </c>
     </row>
     <row r="993">
       <c r="A993" t="str">
-        <v>EWY</v>
-      </c>
-    </row>
-    <row r="994">
-      <c r="A994" t="str">
         <v>SPCX</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A994"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A993"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
watchlist: agregar BRK-B (alta manual desde la app)
</commit_message>
<xml_diff>
--- a/data/tickers.xlsx
+++ b/data/tickers.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A993"/>
+  <dimension ref="A1:A994"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5364,9 +5364,14 @@
         <v>SPCX</v>
       </c>
     </row>
+    <row r="994">
+      <c r="A994" t="str">
+        <v>BRK-B</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A993"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A994"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
watchlist: agregar TQQQ (alta manual desde la app)
</commit_message>
<xml_diff>
--- a/data/tickers.xlsx
+++ b/data/tickers.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A994"/>
+  <dimension ref="A1:A995"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5369,9 +5369,14 @@
         <v>BRK-B</v>
       </c>
     </row>
+    <row r="995">
+      <c r="A995" t="str">
+        <v>TQQQ</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A994"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A995"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
watchlist: agregar GEV (alta manual desde la app)
</commit_message>
<xml_diff>
--- a/data/tickers.xlsx
+++ b/data/tickers.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A995"/>
+  <dimension ref="A1:A996"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5374,9 +5374,14 @@
         <v>TQQQ</v>
       </c>
     </row>
+    <row r="996">
+      <c r="A996" t="str">
+        <v>GEV</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A995"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A996"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
watchlist: agregar DELL (alta manual desde la app)
</commit_message>
<xml_diff>
--- a/data/tickers.xlsx
+++ b/data/tickers.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A996"/>
+  <dimension ref="A1:A997"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5379,9 +5379,14 @@
         <v>GEV</v>
       </c>
     </row>
+    <row r="997">
+      <c r="A997" t="str">
+        <v>DELL</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A996"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A997"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>